<commit_message>
Drop email support line, rename content delivery with delivery dates
Exgrowth's August invoice now has just the content delivery line
(8/17, 8/27x2), dated 8/27, 30,000 yen.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GmiXe9RCHpFsdrbpadPUq2
</commit_message>
<xml_diff>
--- a/invoice_agent/exgrowth_202608.xlsx
+++ b/invoice_agent/exgrowth_202608.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -474,18 +474,18 @@
         </is>
       </c>
       <c r="B2" s="1" t="n">
-        <v>46265</v>
+        <v>46261</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>メール配信サポート6社</t>
+          <t>コンテンツ納品（8/17、8/27×2）</t>
         </is>
       </c>
       <c r="D2" t="n">
         <v>1</v>
       </c>
       <c r="E2" t="n">
-        <v>60000</v>
+        <v>30000</v>
       </c>
       <c r="F2" t="n">
         <v>10</v>
@@ -496,39 +496,7 @@
         </is>
       </c>
       <c r="H2" s="1" t="n">
-        <v>46265</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Exgrowth株式会社</t>
-        </is>
-      </c>
-      <c r="B3" s="1" t="n">
-        <v>46265</v>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>コンテンツ納品</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E3" t="n">
-        <v>30000</v>
-      </c>
-      <c r="F3" t="n">
-        <v>10</v>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>業務委託契約</t>
-        </is>
-      </c>
-      <c r="H3" s="1" t="n">
-        <v>46265</v>
+        <v>46261</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Restore email support line, drop only the "6社" wording
Misread the earlier instruction as removing the whole line; only
the "6社" suffix in the label was meant to go.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GmiXe9RCHpFsdrbpadPUq2
</commit_message>
<xml_diff>
--- a/invoice_agent/exgrowth_202608.xlsx
+++ b/invoice_agent/exgrowth_202608.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -497,6 +497,38 @@
       </c>
       <c r="H2" s="1" t="n">
         <v>46261</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Exgrowth株式会社</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="n">
+        <v>46265</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>メール配信サポート</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" t="n">
+        <v>60000</v>
+      </c>
+      <c r="F3" t="n">
+        <v>10</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>業務委託契約</t>
+        </is>
+      </c>
+      <c r="H3" s="1" t="n">
+        <v>46265</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Exgrowth invoice: delivery date, quantity split, remarks
Delivery date set to 8/31 for both lines, content delivery itemized
as qty 3 x 10,000 yen (matching the three delivery dates), and added
a remarks note on Facebook ads / proposal materials being covered
under email support.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GmiXe9RCHpFsdrbpadPUq2
</commit_message>
<xml_diff>
--- a/invoice_agent/exgrowth_202608.xlsx
+++ b/invoice_agent/exgrowth_202608.xlsx
@@ -482,10 +482,10 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E2" t="n">
-        <v>30000</v>
+        <v>10000</v>
       </c>
       <c r="F2" t="n">
         <v>10</v>
@@ -496,7 +496,12 @@
         </is>
       </c>
       <c r="H2" s="1" t="n">
-        <v>46261</v>
+        <v>46265</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Facebook広告、各種提案資料の作成等につきましては、メール配信サポートの中で実施させていただきました。</t>
+        </is>
       </c>
     </row>
     <row r="3">

</xml_diff>